<commit_message>
feat(cheil): one name per common blank across the six templates
Plan item 1. The same information went by a different blank in each
template ([광고주] / [광고주명], [예산 합계] / [RFP에 적힌 예산 규모],
[제출일] / [보고일] / [날짜]). packages/ui/src/cheil-fields.json now
names the ten common blanks once (campaign, client, brand, period,
budget, target, KPI, team, author, date) with their aliases.

- make_templates.py builds the templates from the dictionary and reopens
  each file: an alias, or a non-common blank appearing twice, fails it
- cheil-fields.ts: lookup by name or alias, the hint the one-call fill
  now sends with a common blank, and a campaign card's values for them
- the six templates regenerated; brief, meeting notes, pitch analysis
  and media plan gained the period/budget/KPI/client rows the card fills
- tests/cheil-fields.test.ts opens the shipped templates and checks them

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/shell/resources/builtin-skills/cheil-media-plan/assets/미디어 플랜.xlsx
+++ b/apps/shell/resources/builtin-skills/cheil-media-plan/assets/미디어 플랜.xlsx
@@ -509,14 +509,21 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>[광고주명] [캠페인명] 미디어 플랜</t>
+          <t>[광고주] [캠페인명] 미디어 플랜</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>작성 [날짜] · [팀명] · 숫자는 매체 견적·합의 자료 기준(출처는 '가정·출처' 시트)</t>
+          <t>작성 [작성일] · [팀명] · 캠페인 기간 [캠페인 기간] · 총예산 [총예산]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>숫자는 매체 견적·합의 자료 기준(출처는 '가정·출처' 시트)</t>
         </is>
       </c>
     </row>

</xml_diff>